<commit_message>
fix: update template-siswa.xlsx with Nama + Blok columns
</commit_message>
<xml_diff>
--- a/public/template-siswa.xlsx
+++ b/public/template-siswa.xlsx
@@ -397,31 +397,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:B4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Nama</v>
       </c>
+      <c r="B1" t="str">
+        <v>Blok</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>Alea</v>
       </c>
+      <c r="B2" t="str">
+        <v>Etan</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
         <v>Budi</v>
       </c>
+      <c r="B3" t="str">
+        <v>Kulon</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
         <v>Citra</v>
       </c>
+      <c r="B4" t="str">
+        <v>Etan</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(kwaru): W logo + E-Waru title + dashboard dynamic counts + 3-blok template
- New W icon (green gradient) for kwaru PWA + header
- Tab title: 'E-Waru' for kwaru, 'Kas Kelas' for kaskelas
- Splash screen: dynamic title + brand for kwaru
- Dashboard: fetch both siswa/guru metrics, show real counts (no hardcoded 11/9)
- Template: 6 examples (3 Etan, 3 Kulon)
</commit_message>
<xml_diff>
--- a/public/template-siswa.xlsx
+++ b/public/template-siswa.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -431,9 +431,33 @@
         <v>Etan</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Dani</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Kulon</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Eka</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Etan</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Farhan</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Kulon</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(kwaru): blok Lainnya + fix logo centering + template 3 blok
- Add 'lainnya' blok option everywhere (DB, API, frontend types, filters, form, Excel parser)
- Fix W logo centering (adjust SVG text position)
- Template: 8 examples (3 Etan, 3 Kulon, 2 Lainnya)
- Form tambah/edit jamaah: 3 blok buttons (Etan/Kulon/Lainnya)
- Filter blok: Semua/Etan/Kulon/Lainnya in Students, Contribution, Recap
</commit_message>
<xml_diff>
--- a/public/template-siswa.xlsx
+++ b/public/template-siswa.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -444,7 +444,7 @@
         <v>Eka</v>
       </c>
       <c r="B6" t="str">
-        <v>Etan</v>
+        <v>Lainnya</v>
       </c>
     </row>
     <row r="7">
@@ -452,12 +452,28 @@
         <v>Farhan</v>
       </c>
       <c r="B7" t="str">
+        <v>Etan</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Gilang</v>
+      </c>
+      <c r="B8" t="str">
         <v>Kulon</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Hana</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Lainnya</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>